<commit_message>
Add camera control feature (on/off + live status)
</commit_message>
<xml_diff>
--- a/database/students_2022-23.xlsx
+++ b/database/students_2022-23.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Face-Recognition-Attendance-System\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3663C3C5-D825-430D-B246-C966B1F56C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08218D1-F745-4BF2-8657-B266D252FDEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27675" yWindow="1125" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="60">
   <si>
     <t>name</t>
   </si>
@@ -190,9 +190,6 @@
   </si>
   <si>
     <t>ibrahimhossain3669@gmail.com</t>
-  </si>
-  <si>
-    <t>3rd Year 2nd Semister</t>
   </si>
   <si>
     <t>Md Abdul Ahad</t>
@@ -301,12 +298,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -321,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -356,9 +359,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -370,6 +370,16 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -589,7 +599,7 @@
   <dimension ref="A1:K1001"/>
   <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.25" customWidth="1"/>
+    <col min="1" max="1" width="22.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.125" style="8" customWidth="1"/>
     <col min="3" max="3" width="10.75" customWidth="1"/>
     <col min="4" max="4" width="30.125" customWidth="1"/>
@@ -600,35 +610,35 @@
     <col min="12" max="26" width="14.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="17" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:11" s="16" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="15"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="20" t="s">
         <v>33</v>
       </c>
       <c r="B2" s="6">
@@ -646,8 +656,8 @@
       <c r="F2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>55</v>
+      <c r="G2" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H2" s="11"/>
       <c r="I2" s="3"/>
@@ -655,7 +665,7 @@
       <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="21" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="6">
@@ -673,8 +683,8 @@
       <c r="F3" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>55</v>
+      <c r="G3" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H3" s="11"/>
       <c r="I3" s="3"/>
@@ -682,7 +692,7 @@
       <c r="K3" s="3"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="20" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="6">
@@ -700,8 +710,8 @@
       <c r="F4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>55</v>
+      <c r="G4" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H4" s="11"/>
       <c r="I4" s="3"/>
@@ -709,7 +719,7 @@
       <c r="K4" s="3"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="21" t="s">
         <v>27</v>
       </c>
       <c r="B5" s="6">
@@ -727,13 +737,13 @@
       <c r="F5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="9" t="s">
-        <v>55</v>
+      <c r="G5" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H5" s="11"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B6" s="6">
@@ -751,13 +761,13 @@
       <c r="F6" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>55</v>
+      <c r="G6" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H6" s="11"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="21" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="6">
@@ -775,13 +785,13 @@
       <c r="F7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>55</v>
+      <c r="G7" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H7" s="11"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="20" t="s">
         <v>30</v>
       </c>
       <c r="B8" s="6">
@@ -799,13 +809,13 @@
       <c r="F8" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="9" t="s">
-        <v>55</v>
+      <c r="G8" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H8" s="11"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="21" t="s">
         <v>34</v>
       </c>
       <c r="B9" s="6">
@@ -823,13 +833,13 @@
       <c r="F9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="9" t="s">
-        <v>55</v>
+      <c r="G9" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H9" s="11"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="20" t="s">
         <v>35</v>
       </c>
       <c r="B10" s="6">
@@ -847,13 +857,13 @@
       <c r="F10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="18" t="s">
-        <v>58</v>
+      <c r="G10" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H10" s="11"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="21" t="s">
         <v>36</v>
       </c>
       <c r="B11" s="6">
@@ -871,13 +881,13 @@
       <c r="F11" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="G11" s="18" t="s">
-        <v>58</v>
+      <c r="G11" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H11" s="11"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="20" t="s">
         <v>37</v>
       </c>
       <c r="B12" s="6">
@@ -895,13 +905,13 @@
       <c r="F12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="18" t="s">
-        <v>58</v>
+      <c r="G12" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H12" s="11"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="21" t="s">
         <v>38</v>
       </c>
       <c r="B13" s="6">
@@ -919,13 +929,13 @@
       <c r="F13" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="G13" s="18" t="s">
-        <v>58</v>
+      <c r="G13" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H13" s="11"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="20" t="s">
         <v>43</v>
       </c>
       <c r="B14" s="6">
@@ -943,13 +953,13 @@
       <c r="F14" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="18" t="s">
-        <v>58</v>
+      <c r="G14" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B15" s="6">
@@ -967,13 +977,13 @@
       <c r="F15" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G15" s="18" t="s">
-        <v>58</v>
+      <c r="G15" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="20" t="s">
         <v>40</v>
       </c>
       <c r="B16" s="6">
@@ -991,13 +1001,13 @@
       <c r="F16" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="18" t="s">
-        <v>58</v>
+      <c r="G16" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="21" t="s">
         <v>41</v>
       </c>
       <c r="B17" s="6">
@@ -1015,13 +1025,13 @@
       <c r="F17" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="G17" s="18" t="s">
-        <v>58</v>
+      <c r="G17" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="20" t="s">
         <v>42</v>
       </c>
       <c r="B18" s="6">
@@ -1039,13 +1049,13 @@
       <c r="F18" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G18" s="18" t="s">
-        <v>58</v>
+      <c r="G18" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="21" t="s">
         <v>44</v>
       </c>
       <c r="B19" s="6">
@@ -1063,13 +1073,13 @@
       <c r="F19" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="18" t="s">
-        <v>58</v>
+      <c r="G19" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H19" s="11"/>
     </row>
     <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="20" t="s">
         <v>47</v>
       </c>
       <c r="B20" s="6">
@@ -1087,13 +1097,13 @@
       <c r="F20" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="G20" s="18" t="s">
-        <v>58</v>
+      <c r="G20" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H20" s="11"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="21" t="s">
         <v>45</v>
       </c>
       <c r="B21" s="6">
@@ -1111,14 +1121,14 @@
       <c r="F21" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="18" t="s">
-        <v>58</v>
+      <c r="G21" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H21" s="11"/>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
-        <v>56</v>
+      <c r="A22" s="20" t="s">
+        <v>55</v>
       </c>
       <c r="B22" s="6">
         <v>220524</v>
@@ -1127,21 +1137,21 @@
         <v>21</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E22" s="6">
         <v>220524</v>
       </c>
       <c r="F22" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G22" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="G22" s="18" t="s">
-        <v>58</v>
-      </c>
       <c r="H22" s="11"/>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="21" t="s">
         <v>46</v>
       </c>
       <c r="B23" s="6">
@@ -1159,13 +1169,13 @@
       <c r="F23" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G23" s="18" t="s">
-        <v>58</v>
+      <c r="G23" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H23" s="11"/>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="20" t="s">
         <v>48</v>
       </c>
       <c r="B24" s="6">
@@ -1183,14 +1193,14 @@
       <c r="F24" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="G24" s="18" t="s">
-        <v>58</v>
+      <c r="G24" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H24" s="11"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>60</v>
+      <c r="A25" s="21" t="s">
+        <v>59</v>
       </c>
       <c r="B25" s="6">
         <v>200536</v>
@@ -1199,16 +1209,16 @@
         <v>25</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E25" s="13">
         <v>200536</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="G25" s="18" t="s">
         <v>58</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>57</v>
       </c>
       <c r="H25" s="11"/>
     </row>

</xml_diff>